<commit_message>
ajuste do código geral
</commit_message>
<xml_diff>
--- a/fgts -reunião.xlsx
+++ b/fgts -reunião.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30602"/>
-  <workbookPr/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
+  <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://mcidades.sharepoint.com/sites/DEMOB/Documentos Compartilhados/AOF/Dados painel/vscode/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="141" documentId="8_{A80E839E-259F-43D5-B3EF-865F9444D52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{77B7EC06-6C49-4512-8525-912E0D2452B7}"/>
+  <xr:revisionPtr revIDLastSave="146" documentId="8_{A80E839E-259F-43D5-B3EF-865F9444D52C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BA463751-6B95-4CBD-9C58-E1E58901C524}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-300" windowWidth="29040" windowHeight="15720" xr2:uid="{FC19E197-98C7-4572-A65B-E1DAE880E8FC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="40" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="47" uniqueCount="26">
   <si>
     <t>REGIÃO</t>
   </si>
@@ -68,12 +68,6 @@
     <t>CONTRATADO REFROTA PÚBLICO</t>
   </si>
   <si>
-    <t>SELEÇÃO A PUBLICAR AVANÇAR</t>
-  </si>
-  <si>
-    <t>SELEÇÃO A PUBLICAR GM PRIVADO</t>
-  </si>
-  <si>
     <t>SELEÇÃO A PUBLICAR REFROTA PRIVADO</t>
   </si>
   <si>
@@ -83,31 +77,13 @@
     <t>SALDO</t>
   </si>
   <si>
-    <t>Centro-Oeste</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> R$                                                      -  </t>
-  </si>
-  <si>
-    <t xml:space="preserve">R$ -   </t>
-  </si>
-  <si>
     <t>Nordeste</t>
   </si>
   <si>
     <t xml:space="preserve"> R$ -   </t>
   </si>
   <si>
-    <t xml:space="preserve"> R$                                                                -  </t>
-  </si>
-  <si>
-    <t xml:space="preserve"> R$                                                                                       -  </t>
-  </si>
-  <si>
     <t>Norte</t>
-  </si>
-  <si>
-    <t xml:space="preserve"> R$                                                               -  </t>
   </si>
   <si>
     <t>Sudeste</t>
@@ -131,6 +107,18 @@
   </si>
   <si>
     <t>- Linha 4:R$1,250 bi</t>
+  </si>
+  <si>
+    <t>A CONTRATAR GM PÚBLICO</t>
+  </si>
+  <si>
+    <t>A CONTRATAR REFROTA PÚBLICO</t>
+  </si>
+  <si>
+    <t>SELEÇÃO A PUBLICAR AVAÇAR</t>
+  </si>
+  <si>
+    <t>Centro - Oeste</t>
   </si>
 </sst>
 </file>
@@ -142,10 +130,16 @@
     <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Aptos Narrow"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -202,7 +196,10 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="14">
+  <dxfs count="15">
+    <dxf>
+      <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+    </dxf>
     <dxf>
       <numFmt numFmtId="34" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
       <fill>
@@ -265,25 +262,24 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8609D132-5F61-49C6-9EE6-034A18AFA5D6}" name="Tabela432" displayName="Tabela432" ref="A1:N7" totalsRowShown="0" headerRowDxfId="13">
-  <autoFilter ref="A1:N7" xr:uid="{8609D132-5F61-49C6-9EE6-034A18AFA5D6}"/>
-  <tableColumns count="14">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{8609D132-5F61-49C6-9EE6-034A18AFA5D6}" name="Tabela432" displayName="Tabela432" ref="A1:O7" totalsRowShown="0" headerRowDxfId="14">
+  <autoFilter ref="A1:O7" xr:uid="{8609D132-5F61-49C6-9EE6-034A18AFA5D6}"/>
+  <tableColumns count="15">
     <tableColumn id="1" xr3:uid="{7F4504F4-2B48-45D0-8044-153C8E8F5641}" name="REGIÃO"/>
-    <tableColumn id="2" xr3:uid="{96A452D1-04FD-4FB1-9B7A-9149B2B32B91}" name="LIMITE" dataDxfId="12"/>
-    <tableColumn id="3" xr3:uid="{DE9EF57E-50D3-4E86-8879-59FB1CDA39D6}" name="A CONTRATAR AVANÇAR" dataDxfId="11"/>
-    <tableColumn id="14" xr3:uid="{3855FB98-CD6C-493A-8706-6B2A217D08AC}" name="A CONTRATAR GM PRIVADO" dataDxfId="10"/>
-    <tableColumn id="11" xr3:uid="{64BE34BE-2D8A-4D18-92CF-862001DAD834}" name="A CONTRATAR REFROTA PRIVADO" dataDxfId="9"/>
-    <tableColumn id="4" xr3:uid="{959B306B-AAE6-41E5-98A1-C189B1C6DD04}" name="CONTRATADO AVANÇAR" dataDxfId="8"/>
-    <tableColumn id="13" xr3:uid="{04BE3386-677B-4927-B182-D83D47640FEB}" name="CONTRATADO GM PÚBLICO" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{45487E33-9D97-4F1F-BBD2-313A2B20FE32}" name="CONTRATADO REFROTA PRIVADO" dataDxfId="6"/>
-    <tableColumn id="17" xr3:uid="{2BFF60E0-6D3D-4C88-862F-3374645E24FA}" name="CONTRATADO REFROTA PÚBLICO" dataDxfId="5"/>
-    <tableColumn id="15" xr3:uid="{E181838B-2884-4788-A770-F1BA7B033365}" name="SELEÇÃO A PUBLICAR AVANÇAR" dataDxfId="4"/>
-    <tableColumn id="6" xr3:uid="{2D888D58-F45D-4EDE-B023-F9A6E9A92B6D}" name="SELEÇÃO A PUBLICAR GM PRIVADO" dataDxfId="3"/>
-    <tableColumn id="18" xr3:uid="{A9760938-0FB5-42B7-98C3-7471395A1291}" name="SELEÇÃO A PUBLICAR REFROTA PRIVADO" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{C619930E-9A6C-4E85-B4DB-D5BE0BC53EEA}" name="VALOR EXECUTADO" dataDxfId="1"/>
-    <tableColumn id="12" xr3:uid="{698399D7-C743-471D-BFA2-DD61CC68FDD2}" name="SALDO" dataDxfId="0">
-      <calculatedColumnFormula>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</calculatedColumnFormula>
-    </tableColumn>
+    <tableColumn id="2" xr3:uid="{96A452D1-04FD-4FB1-9B7A-9149B2B32B91}" name="LIMITE" dataDxfId="13"/>
+    <tableColumn id="3" xr3:uid="{DE9EF57E-50D3-4E86-8879-59FB1CDA39D6}" name="A CONTRATAR AVANÇAR" dataDxfId="12"/>
+    <tableColumn id="14" xr3:uid="{3855FB98-CD6C-493A-8706-6B2A217D08AC}" name="A CONTRATAR GM PRIVADO" dataDxfId="11"/>
+    <tableColumn id="11" xr3:uid="{64BE34BE-2D8A-4D18-92CF-862001DAD834}" name="A CONTRATAR GM PÚBLICO" dataDxfId="10"/>
+    <tableColumn id="4" xr3:uid="{959B306B-AAE6-41E5-98A1-C189B1C6DD04}" name="A CONTRATAR REFROTA PRIVADO" dataDxfId="9"/>
+    <tableColumn id="13" xr3:uid="{04BE3386-677B-4927-B182-D83D47640FEB}" name="A CONTRATAR REFROTA PÚBLICO" dataDxfId="8"/>
+    <tableColumn id="5" xr3:uid="{45487E33-9D97-4F1F-BBD2-313A2B20FE32}" name="SELEÇÃO A PUBLICAR AVAÇAR" dataDxfId="7"/>
+    <tableColumn id="17" xr3:uid="{2BFF60E0-6D3D-4C88-862F-3374645E24FA}" name="SELEÇÃO A PUBLICAR REFROTA PRIVADO" dataDxfId="6"/>
+    <tableColumn id="15" xr3:uid="{E181838B-2884-4788-A770-F1BA7B033365}" name="CONTRATADO AVANÇAR" dataDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{2D888D58-F45D-4EDE-B023-F9A6E9A92B6D}" name="CONTRATADO REFROTA PRIVADO" dataDxfId="4"/>
+    <tableColumn id="18" xr3:uid="{A9760938-0FB5-42B7-98C3-7471395A1291}" name="CONTRATADO REFROTA PÚBLICO" dataDxfId="3"/>
+    <tableColumn id="10" xr3:uid="{C619930E-9A6C-4E85-B4DB-D5BE0BC53EEA}" name="CONTRATADO GM PÚBLICO" dataDxfId="2"/>
+    <tableColumn id="12" xr3:uid="{698399D7-C743-471D-BFA2-DD61CC68FDD2}" name="VALOR EXECUTADO" dataDxfId="1"/>
+    <tableColumn id="7" xr3:uid="{4F34B08A-1B56-4A50-810C-A76E18217A72}" name="SALDO" dataDxfId="0"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
@@ -606,8 +602,8 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3BB739F9-A5E0-4416-9F4A-56B804EE202B}">
-  <dimension ref="A1:N11"/>
-  <sheetFormatPr defaultRowHeight="15"/>
+  <dimension ref="A1:O11"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="25.140625" customWidth="1"/>
     <col min="2" max="2" width="28.42578125" customWidth="1"/>
@@ -619,7 +615,7 @@
     <col min="15" max="15" width="28.5703125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:14">
+    <row r="1" spans="1:15" ht="30" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -633,39 +629,42 @@
         <v>3</v>
       </c>
       <c r="E1" s="2" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="2" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="2" t="s">
+      <c r="G1" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="2" t="s">
+      <c r="K1" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="M1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="K1" s="1" t="s">
+      <c r="N1" s="6" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="O1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="N1" s="6" t="s">
-        <v>13</v>
-      </c>
     </row>
-    <row r="2" spans="1:14">
+    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>14</v>
+        <v>25</v>
       </c>
       <c r="B2" s="7">
         <v>558464000</v>
@@ -674,41 +673,45 @@
         <v>18807909.960000001</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>15</v>
-      </c>
-      <c r="E2" s="7">
-        <v>61750000</v>
+        <v>13</v>
+      </c>
+      <c r="E2" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="F2" s="7">
+        <v>225055000</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H2" s="7">
+        <v>447349233.38999999</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="J2" s="7">
         <v>136099957.27000001</v>
       </c>
-      <c r="G2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="H2" s="7">
+      <c r="K2" s="7">
         <v>124957952.8</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>16</v>
-      </c>
-      <c r="J2" s="7">
-        <v>447349233.38999999</v>
-      </c>
-      <c r="K2" s="3"/>
-      <c r="L2" s="7">
-        <v>153425000</v>
-      </c>
-      <c r="M2" s="7">
+      <c r="L2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="M2" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N2" s="8">
         <v>261057910.06999999</v>
       </c>
-      <c r="N2" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
+      <c r="O2" s="3">
         <v>297406089.93000001</v>
       </c>
     </row>
-    <row r="3" spans="1:14">
+    <row r="3" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="B3" s="7">
         <v>1510048000</v>
@@ -717,235 +720,252 @@
         <v>10763500</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E3" s="7">
+        <v>107679415.69</v>
+      </c>
+      <c r="F3" s="7">
         <v>52250000</v>
       </c>
-      <c r="F3" s="3" t="s">
-        <v>18</v>
-      </c>
       <c r="G3" s="7">
+        <v>95000000</v>
+      </c>
+      <c r="H3" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I3" s="7">
+        <v>23838255</v>
+      </c>
+      <c r="J3" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K3" s="7">
+        <v>264154897.31</v>
+      </c>
+      <c r="L3" s="7">
+        <v>95000000</v>
+      </c>
+      <c r="M3" s="7">
         <v>30587544.359999999</v>
       </c>
-      <c r="H3" s="7">
-        <v>261042697.31</v>
-      </c>
-      <c r="I3" s="7">
-        <v>95000000</v>
-      </c>
-      <c r="J3" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K3" s="3"/>
-      <c r="L3" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M3" s="7">
-        <v>386630241.67000002</v>
-      </c>
       <c r="N3" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
-        <v>1123417758.3299999</v>
+        <v>389742441.67000002</v>
+      </c>
+      <c r="O3" s="3">
+        <v>1120305558.3299999</v>
       </c>
     </row>
-    <row r="4" spans="1:14">
+    <row r="4" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>21</v>
+        <v>14</v>
       </c>
       <c r="B4" s="7">
         <v>456973000</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>22</v>
+        <v>13</v>
       </c>
       <c r="D4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="7">
+        <v>18766300</v>
+      </c>
+      <c r="G4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="H4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="I4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J4" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="K4" s="7">
+        <v>63264813</v>
+      </c>
+      <c r="L4" s="7">
+        <v>67000000</v>
+      </c>
+      <c r="M4" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="N4" s="8">
+        <v>130264813</v>
+      </c>
+      <c r="O4" s="3">
+        <v>326708187</v>
+      </c>
+    </row>
+    <row r="5" spans="1:15" x14ac:dyDescent="0.25">
+      <c r="A5" t="s">
         <v>15</v>
-      </c>
-      <c r="E4" s="7">
-        <v>87166300</v>
-      </c>
-      <c r="F4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="G4" s="3" t="s">
-        <v>18</v>
-      </c>
-      <c r="H4" s="7">
-        <v>63264813</v>
-      </c>
-      <c r="I4" s="7">
-        <v>67000000</v>
-      </c>
-      <c r="J4" s="3" t="s">
-        <v>19</v>
-      </c>
-      <c r="K4" s="3"/>
-      <c r="L4" s="3" t="s">
-        <v>20</v>
-      </c>
-      <c r="M4" s="7">
-        <v>130264813</v>
-      </c>
-      <c r="N4" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
-        <v>326708187</v>
-      </c>
-    </row>
-    <row r="5" spans="1:14">
-      <c r="A5" t="s">
-        <v>23</v>
       </c>
       <c r="B5" s="7">
         <v>2982701000</v>
       </c>
       <c r="C5" s="7">
-        <v>2607387176.6599998</v>
+        <v>1514067726.02</v>
       </c>
       <c r="D5" s="7">
         <v>2789935189.5500002</v>
       </c>
       <c r="E5" s="7">
-        <v>810224910.70000005</v>
+        <v>48264165.210000001</v>
       </c>
       <c r="F5" s="7">
+        <v>749771660.70000005</v>
+      </c>
+      <c r="G5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="H5" s="7">
+        <v>34763862.579999998</v>
+      </c>
+      <c r="I5" s="7" t="s">
+        <v>13</v>
+      </c>
+      <c r="J5" s="7">
         <v>283500000</v>
       </c>
-      <c r="G5" s="7">
-        <v>411660327.30000001</v>
-      </c>
-      <c r="H5" s="7">
-        <v>1791343728.3900001</v>
-      </c>
-      <c r="I5" s="7">
+      <c r="K5" s="7">
+        <v>1805662128.3900001</v>
+      </c>
+      <c r="L5" s="7">
         <v>60312000</v>
       </c>
-      <c r="J5" s="7">
-        <v>34763862.579999998</v>
-      </c>
-      <c r="K5" s="7">
-        <v>1364935189.55</v>
-      </c>
-      <c r="L5" s="3" t="s">
-        <v>20</v>
-      </c>
       <c r="M5" s="7">
-        <v>2546816055.6900001</v>
+        <v>542253272.05999994</v>
       </c>
       <c r="N5" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
-        <v>435884944.30999994</v>
+        <v>2691727400.4499998</v>
+      </c>
+      <c r="O5" s="3">
+        <v>290973599.55000001</v>
       </c>
     </row>
-    <row r="6" spans="1:14">
+    <row r="6" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="B6" s="7">
         <v>891814000</v>
       </c>
       <c r="C6" s="7">
-        <v>311977640.04000002</v>
+        <v>282400103.88</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="E6" s="7">
-        <v>143608999.80000001</v>
+        <v>121260114.94</v>
       </c>
       <c r="F6" s="7">
-        <v>70958485.340000004</v>
+        <v>217975199.80000001</v>
       </c>
       <c r="G6" s="3" t="s">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="H6" s="7">
-        <v>312707369.72000003</v>
+        <v>227440634.56</v>
       </c>
       <c r="I6" s="7">
+        <v>22184400</v>
+      </c>
+      <c r="J6" s="7">
+        <v>72265509.310000002</v>
+      </c>
+      <c r="K6" s="7">
+        <v>325436799.72000003</v>
+      </c>
+      <c r="L6" s="7">
         <v>15600000</v>
       </c>
-      <c r="J6" s="7">
-        <v>227440634.56</v>
-      </c>
-      <c r="K6" s="3"/>
-      <c r="L6" s="7">
-        <v>14753700</v>
-      </c>
-      <c r="M6" s="7">
-        <v>399265855.06</v>
+      <c r="M6" s="7" t="s">
+        <v>13</v>
       </c>
       <c r="N6" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
-        <v>492548144.94</v>
+        <v>413302309.02999997</v>
+      </c>
+      <c r="O6" s="3">
+        <v>478511690.97000003</v>
       </c>
     </row>
-    <row r="7" spans="1:14">
+    <row r="7" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>25</v>
+        <v>17</v>
       </c>
       <c r="B7" s="7">
         <v>6400000000</v>
       </c>
       <c r="C7" s="7">
-        <v>2948936226.6599998</v>
+        <v>1826039239.8599999</v>
       </c>
       <c r="D7" s="7">
         <v>2789935189.5500002</v>
       </c>
       <c r="E7" s="7">
-        <v>1155000210.5</v>
+        <v>277203695.83999997</v>
       </c>
       <c r="F7" s="7">
-        <v>490558442.61000001</v>
+        <v>1263818160.5</v>
       </c>
       <c r="G7" s="7">
-        <v>442247871.66000003</v>
+        <v>95000000</v>
       </c>
       <c r="H7" s="7">
-        <v>2553316561.2199998</v>
+        <v>709553730.52999997</v>
       </c>
       <c r="I7" s="7">
+        <v>46022655</v>
+      </c>
+      <c r="J7" s="7">
+        <v>491865466.57999998</v>
+      </c>
+      <c r="K7" s="7">
+        <v>2583476591.2199998</v>
+      </c>
+      <c r="L7" s="7">
         <v>237912000</v>
       </c>
-      <c r="J7" s="7">
-        <v>709553730.52999997</v>
-      </c>
-      <c r="K7" s="7">
-        <v>1364935189.55</v>
-      </c>
-      <c r="L7" s="7">
-        <v>168178700</v>
-      </c>
       <c r="M7" s="7">
-        <v>3724034875.4899998</v>
+        <v>572840816.41999996</v>
       </c>
       <c r="N7" s="8">
-        <f>Tabela432[[#This Row],[LIMITE]]-Tabela432[[#This Row],[VALOR EXECUTADO]]</f>
-        <v>2675965124.5100002</v>
+        <v>3886094874.2199998</v>
+      </c>
+      <c r="O7" s="3">
+        <v>2513905125.7800002</v>
       </c>
     </row>
-    <row r="9" spans="1:14" s="4" customFormat="1" ht="43.5">
+    <row r="9" spans="1:15" s="4" customFormat="1" ht="45" x14ac:dyDescent="0.25">
       <c r="A9" s="4" t="s">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>27</v>
+        <v>19</v>
       </c>
       <c r="E9" s="5"/>
       <c r="N9" s="5" t="s">
-        <v>28</v>
+        <v>20</v>
       </c>
     </row>
-    <row r="10" spans="1:14">
+    <row r="10" spans="1:15" x14ac:dyDescent="0.25">
       <c r="D10" s="9" t="s">
-        <v>29</v>
+        <v>21</v>
       </c>
     </row>
-    <row r="11" spans="1:14">
+    <row r="11" spans="1:15" x14ac:dyDescent="0.25">
       <c r="C11" s="3"/>
     </row>
   </sheetData>
+  <phoneticPr fontId="1" type="noConversion"/>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">
     <tablePart r:id="rId1"/>
@@ -954,15 +974,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <lcf76f155ced4ddcb4097134ff3c332f xmlns="be150ef9-4f9c-441d-8ced-c7d491dd0c3d">
@@ -971,6 +982,15 @@
     <TaxCatchAll xmlns="402ced5c-caaa-4c89-aae2-d6c39e84cf9c" xsi:nil="true"/>
   </documentManagement>
 </p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1209,13 +1229,39 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED352A8D-207B-4C80-A58D-F51C5A8210E0}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{883DB4C4-CBDC-445E-A9E7-8CFEA139A9F9}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="be150ef9-4f9c-441d-8ced-c7d491dd0c3d"/>
+    <ds:schemaRef ds:uri="402ced5c-caaa-4c89-aae2-d6c39e84cf9c"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{883DB4C4-CBDC-445E-A9E7-8CFEA139A9F9}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{ED352A8D-207B-4C80-A58D-F51C5A8210E0}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33A8BBA2-6947-4BFB-AA72-3704E2BF184D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{33A8BBA2-6947-4BFB-AA72-3704E2BF184D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/2001/XMLSchema"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="be150ef9-4f9c-441d-8ced-c7d491dd0c3d"/>
+    <ds:schemaRef ds:uri="402ced5c-caaa-4c89-aae2-d6c39e84cf9c"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>